<commit_message>
create line regression with using to "torch" renamed line_regression_xlsx.py -> sklearn_line_regression_xlsx.py
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -20,7 +20,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+  <si>
+    <t xml:space="preserve">f1</t>
+  </si>
   <si>
     <t xml:space="preserve">feature2</t>
   </si>
@@ -249,47 +252,62 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="C2" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B3" s="2" t="n">
+    <row r="4" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="n">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="n">
-        <v>5</v>
-      </c>
       <c r="B4" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>8</v>
+        <v>3</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
HSBaded: adaptive columns cheking in tables excel
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -25,7 +25,7 @@
     <t xml:space="preserve">f1</t>
   </si>
   <si>
-    <t xml:space="preserve">feature2</t>
+    <t xml:space="preserve">f2</t>
   </si>
   <si>
     <t xml:space="preserve">target</t>
@@ -285,7 +285,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -307,7 +307,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added stopping criterion: if the weight changes by less than of the specified value
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -255,7 +255,7 @@
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="12.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -266,7 +266,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="12.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="n">
         <v>4</v>
       </c>
@@ -277,7 +277,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="12.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="n">
         <v>7</v>
       </c>
@@ -288,7 +288,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="12.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="n">
         <v>9</v>
       </c>
@@ -299,7 +299,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="12.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="n">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
1 - polinomial degree modification enabled 2 - test values have been added to the graph 3 - duplicates removed 4 - chenged saving of the r2 value
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -268,7 +268,7 @@
     </row>
     <row r="2" customFormat="false" ht="12.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>2</v>
@@ -279,7 +279,7 @@
     </row>
     <row r="3" customFormat="false" ht="12.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>4</v>
@@ -290,7 +290,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>8</v>
@@ -301,7 +301,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
added optimization metod 'ADAM'
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -252,7 +252,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -308,6 +308,17 @@
       </c>
       <c r="C5" s="2" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>